<commit_message>
Refresh live election uploads
</commit_message>
<xml_diff>
--- a/output/Kebbi/results.xlsx
+++ b/output/Kebbi/results.xlsx
@@ -718,7 +718,11 @@
         <v>72741</v>
       </c>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>1781968281058</t>
+        </is>
+      </c>
       <c r="O2" t="n">
         <v>0</v>
       </c>
@@ -739,7 +743,11 @@
         <v>0</v>
       </c>
       <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5317/72045/27d41383-cff0-410c-a5fe-098195598695.jpg</t>
+        </is>
+      </c>
       <c r="X2" t="n">
         <v>0</v>
       </c>
@@ -866,29 +874,43 @@
       <c r="L3" t="n">
         <v>72742</v>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>1781968316511</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>1781968315824</t>
+        </is>
+      </c>
       <c r="O3" t="n">
-        <v>0</v>
+        <v>635</v>
       </c>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="Q3" t="n">
         <v>0</v>
       </c>
-      <c r="R3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>6a36adbc52b6362accb5caac</t>
+        </is>
+      </c>
       <c r="S3" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="T3" t="n">
-        <v>0</v>
+        <v>635</v>
       </c>
       <c r="U3" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5317/72046/a2f6bb12-9341-4e28-a25f-2298352fe2a9.jpg</t>
+        </is>
+      </c>
       <c r="X3" t="n">
         <v>0</v>
       </c>
@@ -905,7 +927,7 @@
         <v>0</v>
       </c>
       <c r="AC3" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="AD3" t="n">
         <v>0</v>
@@ -1016,7 +1038,11 @@
         <v>72743</v>
       </c>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>1781968252886</t>
+        </is>
+      </c>
       <c r="O4" t="n">
         <v>0</v>
       </c>
@@ -1037,7 +1063,11 @@
         <v>0</v>
       </c>
       <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5317/72047/4fa27562-7198-4dd9-b6d9-779812c305fb.jpg</t>
+        </is>
+      </c>
       <c r="X4" t="n">
         <v>0</v>
       </c>
@@ -1463,7 +1493,11 @@
         <v>72746</v>
       </c>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>1781968507479</t>
+        </is>
+      </c>
       <c r="O7" t="n">
         <v>0</v>
       </c>
@@ -1484,7 +1518,11 @@
         <v>0</v>
       </c>
       <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5317/72050/3091af85-94a4-4934-acbd-6f1b41bf97a1.jpg</t>
+        </is>
+      </c>
       <c r="X7" t="n">
         <v>0</v>
       </c>
@@ -2506,7 +2544,11 @@
         <v>154278</v>
       </c>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>1781968313694</t>
+        </is>
+      </c>
       <c r="O14" t="n">
         <v>0</v>
       </c>
@@ -2527,7 +2569,11 @@
         <v>0</v>
       </c>
       <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5317/649565/788dad65-61dc-4617-93b6-c64a094043d2.jpg</t>
+        </is>
+      </c>
       <c r="X14" t="n">
         <v>0</v>
       </c>
@@ -4010,7 +4056,11 @@
         <v>72755</v>
       </c>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>1781970498721</t>
+        </is>
+      </c>
       <c r="O24" t="n">
         <v>0</v>
       </c>
@@ -4031,7 +4081,11 @@
         <v>0</v>
       </c>
       <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5318/72059/8ce17787-f5f0-4320-a4db-4c18fdf73fe3.jpg</t>
+        </is>
+      </c>
       <c r="X24" t="n">
         <v>0</v>
       </c>
@@ -4159,7 +4213,11 @@
         <v>72756</v>
       </c>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>1781968179801</t>
+        </is>
+      </c>
       <c r="O25" t="n">
         <v>0</v>
       </c>
@@ -4180,7 +4238,11 @@
         <v>0</v>
       </c>
       <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5318/72060/607342da-9a1e-49e1-acc0-68a44b47e336.jpg</t>
+        </is>
+      </c>
       <c r="X25" t="n">
         <v>0</v>
       </c>
@@ -7288,7 +7350,11 @@
         <v>154295</v>
       </c>
       <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>1781969590981</t>
+        </is>
+      </c>
       <c r="O46" t="n">
         <v>0</v>
       </c>
@@ -7309,7 +7375,11 @@
         <v>0</v>
       </c>
       <c r="V46" t="inlineStr"/>
-      <c r="W46" t="inlineStr"/>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5319/649582/aecbfd55-d28f-4af0-ac56-9528acd699e6.jpg</t>
+        </is>
+      </c>
       <c r="X46" t="n">
         <v>0</v>
       </c>
@@ -9076,7 +9146,11 @@
         <v>72775</v>
       </c>
       <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>1781969585118</t>
+        </is>
+      </c>
       <c r="O58" t="n">
         <v>0</v>
       </c>
@@ -9097,7 +9171,11 @@
         <v>0</v>
       </c>
       <c r="V58" t="inlineStr"/>
-      <c r="W58" t="inlineStr"/>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5320/72079/2dbf3c18-3c0a-49d1-bdcd-272377b10c9e.jpg</t>
+        </is>
+      </c>
       <c r="X58" t="n">
         <v>0</v>
       </c>
@@ -10566,7 +10644,11 @@
         <v>154306</v>
       </c>
       <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>1781968222024</t>
+        </is>
+      </c>
       <c r="O68" t="n">
         <v>0</v>
       </c>
@@ -10587,7 +10669,11 @@
         <v>0</v>
       </c>
       <c r="V68" t="inlineStr"/>
-      <c r="W68" t="inlineStr"/>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5320/649593/ebc137dd-fc6c-4cbb-b6ab-3d330ead40b6.jpg</t>
+        </is>
+      </c>
       <c r="X68" t="n">
         <v>0</v>
       </c>
@@ -12801,7 +12887,11 @@
         <v>72786</v>
       </c>
       <c r="M83" t="inlineStr"/>
-      <c r="N83" t="inlineStr"/>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>1781968212429</t>
+        </is>
+      </c>
       <c r="O83" t="n">
         <v>0</v>
       </c>
@@ -12822,7 +12912,11 @@
         <v>0</v>
       </c>
       <c r="V83" t="inlineStr"/>
-      <c r="W83" t="inlineStr"/>
+      <c r="W83" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/72090/6de03ebb-b10c-4e79-9dd7-0a9b7d69baf5.jpg</t>
+        </is>
+      </c>
       <c r="X83" t="n">
         <v>0</v>
       </c>
@@ -13545,29 +13639,43 @@
       <c r="L88" t="n">
         <v>72791</v>
       </c>
-      <c r="M88" t="inlineStr"/>
-      <c r="N88" t="inlineStr"/>
+      <c r="M88" t="n">
+        <v>1781968262418</v>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>1781968261818</t>
+        </is>
+      </c>
       <c r="O88" t="n">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="P88" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="Q88" t="n">
         <v>0</v>
       </c>
-      <c r="R88" t="inlineStr"/>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>6a36ad8652b6362accb5c974</t>
+        </is>
+      </c>
       <c r="S88" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="T88" t="n">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="U88" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="V88" t="inlineStr"/>
-      <c r="W88" t="inlineStr"/>
+      <c r="W88" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/72095/2fce395b-3198-43d5-b345-e188fe64f291.jpg</t>
+        </is>
+      </c>
       <c r="X88" t="n">
         <v>0</v>
       </c>
@@ -13584,7 +13692,7 @@
         <v>0</v>
       </c>
       <c r="AC88" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="AD88" t="n">
         <v>0</v>
@@ -13602,7 +13710,7 @@
         <v>0</v>
       </c>
       <c r="AI88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ88" t="n">
         <v>0</v>
@@ -13695,7 +13803,11 @@
         <v>72792</v>
       </c>
       <c r="M89" t="inlineStr"/>
-      <c r="N89" t="inlineStr"/>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>1781968146463</t>
+        </is>
+      </c>
       <c r="O89" t="n">
         <v>0</v>
       </c>
@@ -13716,7 +13828,11 @@
         <v>0</v>
       </c>
       <c r="V89" t="inlineStr"/>
-      <c r="W89" t="inlineStr"/>
+      <c r="W89" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/72096/9b34d24c-5b49-443c-99d0-cbf017ece934.jpg</t>
+        </is>
+      </c>
       <c r="X89" t="n">
         <v>0</v>
       </c>
@@ -13844,7 +13960,11 @@
         <v>72793</v>
       </c>
       <c r="M90" t="inlineStr"/>
-      <c r="N90" t="inlineStr"/>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>1781968182751</t>
+        </is>
+      </c>
       <c r="O90" t="n">
         <v>0</v>
       </c>
@@ -13865,7 +13985,11 @@
         <v>0</v>
       </c>
       <c r="V90" t="inlineStr"/>
-      <c r="W90" t="inlineStr"/>
+      <c r="W90" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/72097/c0356c10-387b-42f0-ae89-fc1546eb7e4e.jpg</t>
+        </is>
+      </c>
       <c r="X90" t="n">
         <v>0</v>
       </c>
@@ -14440,7 +14564,11 @@
         <v>154314</v>
       </c>
       <c r="M94" t="inlineStr"/>
-      <c r="N94" t="inlineStr"/>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>1781968194487</t>
+        </is>
+      </c>
       <c r="O94" t="n">
         <v>0</v>
       </c>
@@ -14461,7 +14589,11 @@
         <v>0</v>
       </c>
       <c r="V94" t="inlineStr"/>
-      <c r="W94" t="inlineStr"/>
+      <c r="W94" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/649603/38ca1365-f145-4cf2-a9f9-069739f81d8f.jpg</t>
+        </is>
+      </c>
       <c r="X94" t="n">
         <v>0</v>
       </c>
@@ -15334,7 +15466,11 @@
         <v>154320</v>
       </c>
       <c r="M100" t="inlineStr"/>
-      <c r="N100" t="inlineStr"/>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>1781968189364</t>
+        </is>
+      </c>
       <c r="O100" t="n">
         <v>0</v>
       </c>
@@ -15355,7 +15491,11 @@
         <v>0</v>
       </c>
       <c r="V100" t="inlineStr"/>
-      <c r="W100" t="inlineStr"/>
+      <c r="W100" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/649609/57add274-98e2-47f0-ba93-9903be92a307.jpg</t>
+        </is>
+      </c>
       <c r="X100" t="n">
         <v>0</v>
       </c>
@@ -15483,7 +15623,11 @@
         <v>154321</v>
       </c>
       <c r="M101" t="inlineStr"/>
-      <c r="N101" t="inlineStr"/>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>1781968156422</t>
+        </is>
+      </c>
       <c r="O101" t="n">
         <v>0</v>
       </c>
@@ -15504,7 +15648,11 @@
         <v>0</v>
       </c>
       <c r="V101" t="inlineStr"/>
-      <c r="W101" t="inlineStr"/>
+      <c r="W101" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/649610/9cdd1a94-ee88-4f76-8fba-c07079f11ba9.jpg</t>
+        </is>
+      </c>
       <c r="X101" t="n">
         <v>0</v>
       </c>
@@ -16228,7 +16376,11 @@
         <v>154326</v>
       </c>
       <c r="M106" t="inlineStr"/>
-      <c r="N106" t="inlineStr"/>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>1781968254026</t>
+        </is>
+      </c>
       <c r="O106" t="n">
         <v>0</v>
       </c>
@@ -16249,7 +16401,11 @@
         <v>0</v>
       </c>
       <c r="V106" t="inlineStr"/>
-      <c r="W106" t="inlineStr"/>
+      <c r="W106" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/649615/8b8fc329-5147-48b3-87e8-1b28aa88993e.jpg</t>
+        </is>
+      </c>
       <c r="X106" t="n">
         <v>0</v>
       </c>
@@ -16824,7 +16980,11 @@
         <v>154330</v>
       </c>
       <c r="M110" t="inlineStr"/>
-      <c r="N110" t="inlineStr"/>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>1781968174850</t>
+        </is>
+      </c>
       <c r="O110" t="n">
         <v>0</v>
       </c>
@@ -16845,7 +17005,11 @@
         <v>0</v>
       </c>
       <c r="V110" t="inlineStr"/>
-      <c r="W110" t="inlineStr"/>
+      <c r="W110" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/649619/8488e8f6-422d-4a92-be0c-17f5a44b9daa.jpg</t>
+        </is>
+      </c>
       <c r="X110" t="n">
         <v>0</v>
       </c>
@@ -17569,7 +17733,11 @@
         <v>154335</v>
       </c>
       <c r="M115" t="inlineStr"/>
-      <c r="N115" t="inlineStr"/>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>1781969587582</t>
+        </is>
+      </c>
       <c r="O115" t="n">
         <v>0</v>
       </c>
@@ -17590,7 +17758,11 @@
         <v>0</v>
       </c>
       <c r="V115" t="inlineStr"/>
-      <c r="W115" t="inlineStr"/>
+      <c r="W115" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/649624/b55022e4-a4c0-45c1-a748-051a36676190.jpg</t>
+        </is>
+      </c>
       <c r="X115" t="n">
         <v>0</v>
       </c>
@@ -18165,7 +18337,11 @@
         <v>154339</v>
       </c>
       <c r="M119" t="inlineStr"/>
-      <c r="N119" t="inlineStr"/>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>1781969225845</t>
+        </is>
+      </c>
       <c r="O119" t="n">
         <v>0</v>
       </c>
@@ -18186,7 +18362,11 @@
         <v>0</v>
       </c>
       <c r="V119" t="inlineStr"/>
-      <c r="W119" t="inlineStr"/>
+      <c r="W119" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/649628/33027a4f-5cca-4b2d-bd3c-8787dafcb35f.jpg</t>
+        </is>
+      </c>
       <c r="X119" t="n">
         <v>0</v>
       </c>
@@ -18611,29 +18791,43 @@
       <c r="L122" t="n">
         <v>154342</v>
       </c>
-      <c r="M122" t="inlineStr"/>
-      <c r="N122" t="inlineStr"/>
+      <c r="M122" t="n">
+        <v>1781968146860</v>
+      </c>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>1781968146231</t>
+        </is>
+      </c>
       <c r="O122" t="n">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="P122" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="Q122" t="n">
-        <v>0</v>
-      </c>
-      <c r="R122" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="R122" t="inlineStr">
+        <is>
+          <t>6a36ad1252b6362accb5c5c0</t>
+        </is>
+      </c>
       <c r="S122" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="T122" t="n">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="U122" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="V122" t="inlineStr"/>
-      <c r="W122" t="inlineStr"/>
+      <c r="W122" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/649631/3a6e3ced-d974-48d0-b5f9-779f0faba39c.jpg</t>
+        </is>
+      </c>
       <c r="X122" t="n">
         <v>0</v>
       </c>
@@ -18650,7 +18844,7 @@
         <v>0</v>
       </c>
       <c r="AC122" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="AD122" t="n">
         <v>0</v>
@@ -18668,7 +18862,7 @@
         <v>0</v>
       </c>
       <c r="AI122" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AJ122" t="n">
         <v>0</v>
@@ -18761,7 +18955,11 @@
         <v>72797</v>
       </c>
       <c r="M123" t="inlineStr"/>
-      <c r="N123" t="inlineStr"/>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>1781968195066</t>
+        </is>
+      </c>
       <c r="O123" t="n">
         <v>0</v>
       </c>
@@ -18782,7 +18980,11 @@
         <v>0</v>
       </c>
       <c r="V123" t="inlineStr"/>
-      <c r="W123" t="inlineStr"/>
+      <c r="W123" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/72101/aed6f9f9-e9ac-41c6-8c7c-dff0732f535b.jpg</t>
+        </is>
+      </c>
       <c r="X123" t="n">
         <v>0</v>
       </c>
@@ -19506,7 +19708,11 @@
         <v>72802</v>
       </c>
       <c r="M128" t="inlineStr"/>
-      <c r="N128" t="inlineStr"/>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>1781968193424</t>
+        </is>
+      </c>
       <c r="O128" t="n">
         <v>0</v>
       </c>
@@ -19527,7 +19733,11 @@
         <v>0</v>
       </c>
       <c r="V128" t="inlineStr"/>
-      <c r="W128" t="inlineStr"/>
+      <c r="W128" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/72106/3bcffcde-7421-424c-ad32-e746c01f6dfe.jpg</t>
+        </is>
+      </c>
       <c r="X128" t="n">
         <v>0</v>
       </c>
@@ -20549,7 +20759,11 @@
         <v>154346</v>
       </c>
       <c r="M135" t="inlineStr"/>
-      <c r="N135" t="inlineStr"/>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>1781970500848</t>
+        </is>
+      </c>
       <c r="O135" t="n">
         <v>0</v>
       </c>
@@ -20570,7 +20784,11 @@
         <v>0</v>
       </c>
       <c r="V135" t="inlineStr"/>
-      <c r="W135" t="inlineStr"/>
+      <c r="W135" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/649635/7f0b0537-5554-48a2-8620-fedf7ed7c285.jpg</t>
+        </is>
+      </c>
       <c r="X135" t="n">
         <v>0</v>
       </c>
@@ -22486,7 +22704,11 @@
         <v>154359</v>
       </c>
       <c r="M148" t="inlineStr"/>
-      <c r="N148" t="inlineStr"/>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>1781968865745</t>
+        </is>
+      </c>
       <c r="O148" t="n">
         <v>0</v>
       </c>
@@ -22507,7 +22729,11 @@
         <v>0</v>
       </c>
       <c r="V148" t="inlineStr"/>
-      <c r="W148" t="inlineStr"/>
+      <c r="W148" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/649648/b23da184-efa9-49ae-92eb-a2ecccf23c8b.jpg</t>
+        </is>
+      </c>
       <c r="X148" t="n">
         <v>0</v>
       </c>
@@ -22783,29 +23009,43 @@
       <c r="L150" t="n">
         <v>154361</v>
       </c>
-      <c r="M150" t="inlineStr"/>
-      <c r="N150" t="inlineStr"/>
+      <c r="M150" t="n">
+        <v>1781969591533</v>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>1781969590981</t>
+        </is>
+      </c>
       <c r="O150" t="n">
-        <v>0</v>
+        <v>748</v>
       </c>
       <c r="P150" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="Q150" t="n">
         <v>0</v>
       </c>
-      <c r="R150" t="inlineStr"/>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>6a36b2b752b6362accb5ccb6</t>
+        </is>
+      </c>
       <c r="S150" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="T150" t="n">
-        <v>0</v>
+        <v>374</v>
       </c>
       <c r="U150" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="V150" t="inlineStr"/>
-      <c r="W150" t="inlineStr"/>
+      <c r="W150" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/649650/e86fa249-37e6-4935-8fe9-f228a050fc10.jpg</t>
+        </is>
+      </c>
       <c r="X150" t="n">
         <v>0</v>
       </c>
@@ -22822,7 +23062,7 @@
         <v>0</v>
       </c>
       <c r="AC150" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="AD150" t="n">
         <v>0</v>
@@ -22840,7 +23080,7 @@
         <v>0</v>
       </c>
       <c r="AI150" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ150" t="n">
         <v>0</v>
@@ -22933,7 +23173,11 @@
         <v>72806</v>
       </c>
       <c r="M151" t="inlineStr"/>
-      <c r="N151" t="inlineStr"/>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>1781970513318</t>
+        </is>
+      </c>
       <c r="O151" t="n">
         <v>0</v>
       </c>
@@ -22954,7 +23198,11 @@
         <v>0</v>
       </c>
       <c r="V151" t="inlineStr"/>
-      <c r="W151" t="inlineStr"/>
+      <c r="W151" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5323/72110/59975ccd-7c7e-4047-8756-bfb53ca4ae56.jpg</t>
+        </is>
+      </c>
       <c r="X151" t="n">
         <v>0</v>
       </c>
@@ -23082,7 +23330,11 @@
         <v>72807</v>
       </c>
       <c r="M152" t="inlineStr"/>
-      <c r="N152" t="inlineStr"/>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>1781968291833</t>
+        </is>
+      </c>
       <c r="O152" t="n">
         <v>0</v>
       </c>
@@ -23103,7 +23355,11 @@
         <v>0</v>
       </c>
       <c r="V152" t="inlineStr"/>
-      <c r="W152" t="inlineStr"/>
+      <c r="W152" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5323/72111/90063bf8-9584-4e4d-a710-2b30f45ad67d.jpg</t>
+        </is>
+      </c>
       <c r="X152" t="n">
         <v>0</v>
       </c>
@@ -23678,7 +23934,11 @@
         <v>72811</v>
       </c>
       <c r="M156" t="inlineStr"/>
-      <c r="N156" t="inlineStr"/>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>1781968296517</t>
+        </is>
+      </c>
       <c r="O156" t="n">
         <v>0</v>
       </c>
@@ -23699,7 +23959,11 @@
         <v>0</v>
       </c>
       <c r="V156" t="inlineStr"/>
-      <c r="W156" t="inlineStr"/>
+      <c r="W156" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5323/72115/e587a5ae-d607-4427-afc8-730d18d311ec.jpg</t>
+        </is>
+      </c>
       <c r="X156" t="n">
         <v>0</v>
       </c>
@@ -24125,7 +24389,11 @@
         <v>154363</v>
       </c>
       <c r="M159" t="inlineStr"/>
-      <c r="N159" t="inlineStr"/>
+      <c r="N159" t="inlineStr">
+        <is>
+          <t>1781968180110</t>
+        </is>
+      </c>
       <c r="O159" t="n">
         <v>0</v>
       </c>
@@ -24146,7 +24414,11 @@
         <v>0</v>
       </c>
       <c r="V159" t="inlineStr"/>
-      <c r="W159" t="inlineStr"/>
+      <c r="W159" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5323/649652/efd6c995-fd91-4731-86f9-bce618aeb6de.jpg</t>
+        </is>
+      </c>
       <c r="X159" t="n">
         <v>0</v>
       </c>
@@ -26211,7 +26483,11 @@
         <v>154368</v>
       </c>
       <c r="M173" t="inlineStr"/>
-      <c r="N173" t="inlineStr"/>
+      <c r="N173" t="inlineStr">
+        <is>
+          <t>1781969589958</t>
+        </is>
+      </c>
       <c r="O173" t="n">
         <v>0</v>
       </c>
@@ -26232,7 +26508,11 @@
         <v>0</v>
       </c>
       <c r="V173" t="inlineStr"/>
-      <c r="W173" t="inlineStr"/>
+      <c r="W173" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5324/649657/f40810c7-32f5-4a9a-ac97-962fe16274cc.jpg</t>
+        </is>
+      </c>
       <c r="X173" t="n">
         <v>0</v>
       </c>
@@ -26360,7 +26640,11 @@
         <v>154369</v>
       </c>
       <c r="M174" t="inlineStr"/>
-      <c r="N174" t="inlineStr"/>
+      <c r="N174" t="inlineStr">
+        <is>
+          <t>1781970495058</t>
+        </is>
+      </c>
       <c r="O174" t="n">
         <v>0</v>
       </c>
@@ -26381,7 +26665,11 @@
         <v>0</v>
       </c>
       <c r="V174" t="inlineStr"/>
-      <c r="W174" t="inlineStr"/>
+      <c r="W174" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5324/649658/3f72ba11-2c82-45dd-87c5-96d03d89795b.jpg</t>
+        </is>
+      </c>
       <c r="X174" t="n">
         <v>0</v>
       </c>
@@ -26658,7 +26946,11 @@
         <v>154371</v>
       </c>
       <c r="M176" t="inlineStr"/>
-      <c r="N176" t="inlineStr"/>
+      <c r="N176" t="inlineStr">
+        <is>
+          <t>1781968206049</t>
+        </is>
+      </c>
       <c r="O176" t="n">
         <v>0</v>
       </c>
@@ -26679,7 +26971,11 @@
         <v>0</v>
       </c>
       <c r="V176" t="inlineStr"/>
-      <c r="W176" t="inlineStr"/>
+      <c r="W176" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5324/675487/b7f28406-55de-40df-ba16-287574920402.jpg</t>
+        </is>
+      </c>
       <c r="X176" t="n">
         <v>0</v>
       </c>
@@ -27403,7 +27699,11 @@
         <v>72825</v>
       </c>
       <c r="M181" t="inlineStr"/>
-      <c r="N181" t="inlineStr"/>
+      <c r="N181" t="inlineStr">
+        <is>
+          <t>1781968259022</t>
+        </is>
+      </c>
       <c r="O181" t="n">
         <v>0</v>
       </c>
@@ -27424,7 +27724,11 @@
         <v>0</v>
       </c>
       <c r="V181" t="inlineStr"/>
-      <c r="W181" t="inlineStr"/>
+      <c r="W181" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5325/72129/f52c739e-2547-42a4-b71d-2e52f593c0b5.jpg</t>
+        </is>
+      </c>
       <c r="X181" t="n">
         <v>0</v>
       </c>
@@ -27552,7 +27856,11 @@
         <v>72826</v>
       </c>
       <c r="M182" t="inlineStr"/>
-      <c r="N182" t="inlineStr"/>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>1781968306441</t>
+        </is>
+      </c>
       <c r="O182" t="n">
         <v>0</v>
       </c>
@@ -27573,7 +27881,11 @@
         <v>0</v>
       </c>
       <c r="V182" t="inlineStr"/>
-      <c r="W182" t="inlineStr"/>
+      <c r="W182" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5325/72130/d7e635f0-44b7-43eb-b027-23ade70a3830.jpg</t>
+        </is>
+      </c>
       <c r="X182" t="n">
         <v>0</v>
       </c>
@@ -27701,7 +28013,11 @@
         <v>72827</v>
       </c>
       <c r="M183" t="inlineStr"/>
-      <c r="N183" t="inlineStr"/>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>1781968215536</t>
+        </is>
+      </c>
       <c r="O183" t="n">
         <v>0</v>
       </c>
@@ -27722,7 +28038,11 @@
         <v>0</v>
       </c>
       <c r="V183" t="inlineStr"/>
-      <c r="W183" t="inlineStr"/>
+      <c r="W183" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5325/72131/05c61c65-797d-4610-b67d-2b704bd3151b.jpg</t>
+        </is>
+      </c>
       <c r="X183" t="n">
         <v>0</v>
       </c>
@@ -27850,7 +28170,11 @@
         <v>72828</v>
       </c>
       <c r="M184" t="inlineStr"/>
-      <c r="N184" t="inlineStr"/>
+      <c r="N184" t="inlineStr">
+        <is>
+          <t>1781968301147</t>
+        </is>
+      </c>
       <c r="O184" t="n">
         <v>0</v>
       </c>
@@ -27871,7 +28195,11 @@
         <v>0</v>
       </c>
       <c r="V184" t="inlineStr"/>
-      <c r="W184" t="inlineStr"/>
+      <c r="W184" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5325/72132/f7244041-4d21-4998-80aa-715250ffbf58.jpg</t>
+        </is>
+      </c>
       <c r="X184" t="n">
         <v>0</v>
       </c>
@@ -30665,22 +30993,22 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>200</v>
+        <v>835</v>
       </c>
       <c r="E2" t="n">
-        <v>31</v>
+        <v>85</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>31</v>
+        <v>85</v>
       </c>
       <c r="H2" t="n">
-        <v>200</v>
+        <v>835</v>
       </c>
       <c r="I2" t="n">
-        <v>31</v>
+        <v>85</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -30698,7 +31026,7 @@
         <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>27</v>
+        <v>81</v>
       </c>
       <c r="P2" t="n">
         <v>0</v>
@@ -31081,22 +31409,22 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -31114,7 +31442,7 @@
         <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="P6" t="n">
         <v>0</v>
@@ -31132,7 +31460,7 @@
         <v>0</v>
       </c>
       <c r="U6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="V6" t="n">
         <v>0</v>
@@ -31185,22 +31513,22 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>748</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>374</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -31218,7 +31546,7 @@
         <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="P7" t="n">
         <v>0</v>
@@ -31236,7 +31564,7 @@
         <v>0</v>
       </c>
       <c r="U7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V7" t="n">
         <v>0</v>
@@ -31871,22 +32199,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>3083</v>
       </c>
       <c r="D2" t="n">
-        <v>31</v>
+        <v>184</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F2" t="n">
-        <v>31</v>
+        <v>182</v>
       </c>
       <c r="G2" t="n">
-        <v>200</v>
+        <v>2709</v>
       </c>
       <c r="H2" t="n">
-        <v>31</v>
+        <v>178</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -31904,7 +32232,7 @@
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>27</v>
+        <v>169</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -31922,7 +32250,7 @@
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
@@ -32131,22 +32459,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>200</v>
+        <v>3083</v>
       </c>
       <c r="C2" t="n">
-        <v>31</v>
+        <v>184</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>31</v>
+        <v>182</v>
       </c>
       <c r="F2" t="n">
-        <v>200</v>
+        <v>2709</v>
       </c>
       <c r="G2" t="n">
-        <v>31</v>
+        <v>178</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -32164,7 +32492,7 @@
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>27</v>
+        <v>169</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
@@ -32182,7 +32510,7 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="T2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Auto-refresh live election results 2026-06-20 12:42:49
</commit_message>
<xml_diff>
--- a/output/Kebbi/results.xlsx
+++ b/output/Kebbi/results.xlsx
@@ -1195,7 +1195,11 @@
         <v>72744</v>
       </c>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>1781976938217</t>
+        </is>
+      </c>
       <c r="O5" t="n">
         <v>0</v>
       </c>
@@ -1216,7 +1220,11 @@
         <v>0</v>
       </c>
       <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5317/72048/efb9ce1b-c452-4cf4-8cc8-f22ff0a27180.jpg</t>
+        </is>
+      </c>
       <c r="X5" t="n">
         <v>0</v>
       </c>
@@ -1344,7 +1352,11 @@
         <v>72745</v>
       </c>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>1781977070325</t>
+        </is>
+      </c>
       <c r="O6" t="n">
         <v>0</v>
       </c>
@@ -1365,7 +1377,11 @@
         <v>0</v>
       </c>
       <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5317/72049/61e4c2c5-8f81-4a0f-87ab-593b3a38e17b.jpg</t>
+        </is>
+      </c>
       <c r="X6" t="n">
         <v>0</v>
       </c>
@@ -1807,7 +1823,11 @@
         <v>72748</v>
       </c>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>1781977001150</t>
+        </is>
+      </c>
       <c r="O9" t="n">
         <v>0</v>
       </c>
@@ -1828,7 +1848,11 @@
         <v>0</v>
       </c>
       <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5317/72052/434f0e4f-5290-4465-a6e8-3dbc21657476.jpg</t>
+        </is>
+      </c>
       <c r="X9" t="n">
         <v>0</v>
       </c>
@@ -1956,7 +1980,11 @@
         <v>72749</v>
       </c>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>1781976785520</t>
+        </is>
+      </c>
       <c r="O10" t="n">
         <v>0</v>
       </c>
@@ -1977,7 +2005,11 @@
         <v>0</v>
       </c>
       <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5317/72053/ee6d79f4-f721-48d8-b8d9-26a5df9b2749.jpg</t>
+        </is>
+      </c>
       <c r="X10" t="n">
         <v>0</v>
       </c>
@@ -2105,7 +2137,11 @@
         <v>72750</v>
       </c>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>1781977038858</t>
+        </is>
+      </c>
       <c r="O11" t="n">
         <v>0</v>
       </c>
@@ -2126,7 +2162,11 @@
         <v>0</v>
       </c>
       <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5317/72054/3852d098-6d82-4dd0-8728-2ab7dd89ce5e.jpg</t>
+        </is>
+      </c>
       <c r="X11" t="n">
         <v>0</v>
       </c>
@@ -2874,7 +2914,11 @@
         <v>154280</v>
       </c>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>1781976770698</t>
+        </is>
+      </c>
       <c r="O16" t="n">
         <v>0</v>
       </c>
@@ -2895,7 +2939,11 @@
         <v>0</v>
       </c>
       <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5317/649567/7e036c0f-6bb2-46f2-99bc-9feb71472910.jpg</t>
+        </is>
+      </c>
       <c r="X16" t="n">
         <v>0</v>
       </c>
@@ -3321,7 +3369,11 @@
         <v>154283</v>
       </c>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>1781976881304</t>
+        </is>
+      </c>
       <c r="O19" t="n">
         <v>0</v>
       </c>
@@ -3342,7 +3394,11 @@
         <v>0</v>
       </c>
       <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr"/>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5317/649570/06d94cca-44ad-4a08-8b73-c3a4b2e7f714.jpg</t>
+        </is>
+      </c>
       <c r="X19" t="n">
         <v>0</v>
       </c>
@@ -3947,7 +4003,11 @@
         <v>72754</v>
       </c>
       <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>1781976936330</t>
+        </is>
+      </c>
       <c r="O23" t="n">
         <v>0</v>
       </c>
@@ -3968,7 +4028,11 @@
         <v>0</v>
       </c>
       <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr"/>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5318/72058/cd8d82b8-a24c-40bc-89a1-9bc0c1be0d6a.jpg</t>
+        </is>
+      </c>
       <c r="X23" t="n">
         <v>0</v>
       </c>
@@ -4716,7 +4780,11 @@
         <v>72759</v>
       </c>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>1781976901539</t>
+        </is>
+      </c>
       <c r="O28" t="n">
         <v>0</v>
       </c>
@@ -4737,7 +4805,11 @@
         <v>0</v>
       </c>
       <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5318/72063/1d3cdcf4-2d83-4a35-b5f1-8ba842fa326e.jpg</t>
+        </is>
+      </c>
       <c r="X28" t="n">
         <v>0</v>
       </c>
@@ -5014,7 +5086,11 @@
         <v>72761</v>
       </c>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>1781977093861</t>
+        </is>
+      </c>
       <c r="O30" t="n">
         <v>0</v>
       </c>
@@ -5035,7 +5111,11 @@
         <v>0</v>
       </c>
       <c r="V30" t="inlineStr"/>
-      <c r="W30" t="inlineStr"/>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5318/72065/5c0a2c79-baca-4670-8e86-129aa7170122.jpg</t>
+        </is>
+      </c>
       <c r="X30" t="n">
         <v>0</v>
       </c>
@@ -5163,7 +5243,11 @@
         <v>72762</v>
       </c>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>1781976792125</t>
+        </is>
+      </c>
       <c r="O31" t="n">
         <v>0</v>
       </c>
@@ -5184,7 +5268,11 @@
         <v>0</v>
       </c>
       <c r="V31" t="inlineStr"/>
-      <c r="W31" t="inlineStr"/>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5318/72066/9060523a-1586-4992-bc5f-ba49b7fba3ea.jpg</t>
+        </is>
+      </c>
       <c r="X31" t="n">
         <v>0</v>
       </c>
@@ -5312,7 +5400,11 @@
         <v>154286</v>
       </c>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>1781977004094</t>
+        </is>
+      </c>
       <c r="O32" t="n">
         <v>0</v>
       </c>
@@ -5333,7 +5425,11 @@
         <v>0</v>
       </c>
       <c r="V32" t="inlineStr"/>
-      <c r="W32" t="inlineStr"/>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5318/649573/171e417d-ec1a-4845-8a56-b4ecd80d7ee1.jpg</t>
+        </is>
+      </c>
       <c r="X32" t="n">
         <v>0</v>
       </c>
@@ -5461,7 +5557,11 @@
         <v>154287</v>
       </c>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>1781976811127</t>
+        </is>
+      </c>
       <c r="O33" t="n">
         <v>0</v>
       </c>
@@ -5482,7 +5582,11 @@
         <v>0</v>
       </c>
       <c r="V33" t="inlineStr"/>
-      <c r="W33" t="inlineStr"/>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5318/649574/d678ca5a-9202-4162-9906-0afae8e01bf7.jpg</t>
+        </is>
+      </c>
       <c r="X33" t="n">
         <v>0</v>
       </c>
@@ -5767,7 +5871,11 @@
         <v>154289</v>
       </c>
       <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>1781977117302</t>
+        </is>
+      </c>
       <c r="O35" t="n">
         <v>0</v>
       </c>
@@ -5788,7 +5896,11 @@
         <v>0</v>
       </c>
       <c r="V35" t="inlineStr"/>
-      <c r="W35" t="inlineStr"/>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5318/649576/cc618dba-655a-48a1-8e7b-6144a2ca2803.jpg</t>
+        </is>
+      </c>
       <c r="X35" t="n">
         <v>0</v>
       </c>
@@ -6362,29 +6474,43 @@
       <c r="L39" t="n">
         <v>72763</v>
       </c>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
+      <c r="M39" t="n">
+        <v>1781976859255</v>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>1781976858595</t>
+        </is>
+      </c>
       <c r="O39" t="n">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="P39" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="Q39" t="n">
-        <v>0</v>
-      </c>
-      <c r="R39" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>6a36cf1a370583337b6e715d</t>
+        </is>
+      </c>
       <c r="S39" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="T39" t="n">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="U39" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="V39" t="inlineStr"/>
-      <c r="W39" t="inlineStr"/>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5319/72067/f6a04854-c2b8-4b98-83c6-b7f18f009ca2.jpg</t>
+        </is>
+      </c>
       <c r="X39" t="n">
         <v>0</v>
       </c>
@@ -6401,7 +6527,7 @@
         <v>0</v>
       </c>
       <c r="AC39" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="AD39" t="n">
         <v>0</v>
@@ -6512,7 +6638,11 @@
         <v>72764</v>
       </c>
       <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>1781976898665</t>
+        </is>
+      </c>
       <c r="O40" t="n">
         <v>0</v>
       </c>
@@ -6533,7 +6663,11 @@
         <v>0</v>
       </c>
       <c r="V40" t="inlineStr"/>
-      <c r="W40" t="inlineStr"/>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5319/72068/d4adeec0-46b0-403d-b709-38bd0929a9ad.jpg</t>
+        </is>
+      </c>
       <c r="X40" t="n">
         <v>0</v>
       </c>
@@ -7281,7 +7415,11 @@
         <v>154294</v>
       </c>
       <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>1781976919683</t>
+        </is>
+      </c>
       <c r="O45" t="n">
         <v>0</v>
       </c>
@@ -7302,7 +7440,11 @@
         <v>0</v>
       </c>
       <c r="V45" t="inlineStr"/>
-      <c r="W45" t="inlineStr"/>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5319/649581/a27689ac-17fa-46a8-a5b2-ebfb0d9ea9ef.jpg</t>
+        </is>
+      </c>
       <c r="X45" t="n">
         <v>0</v>
       </c>
@@ -7587,7 +7729,11 @@
         <v>154296</v>
       </c>
       <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>1781977067972</t>
+        </is>
+      </c>
       <c r="O47" t="n">
         <v>0</v>
       </c>
@@ -7608,7 +7754,11 @@
         <v>0</v>
       </c>
       <c r="V47" t="inlineStr"/>
-      <c r="W47" t="inlineStr"/>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5319/649583/56a88955-6bb0-47d0-b22b-3cfe4790d475.jpg</t>
+        </is>
+      </c>
       <c r="X47" t="n">
         <v>0</v>
       </c>
@@ -7736,7 +7886,11 @@
         <v>154297</v>
       </c>
       <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>1781977018668</t>
+        </is>
+      </c>
       <c r="O48" t="n">
         <v>0</v>
       </c>
@@ -7757,7 +7911,11 @@
         <v>0</v>
       </c>
       <c r="V48" t="inlineStr"/>
-      <c r="W48" t="inlineStr"/>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5319/649584/8d78ce20-3651-45bd-baf1-8de0a716fc1e.jpg</t>
+        </is>
+      </c>
       <c r="X48" t="n">
         <v>0</v>
       </c>
@@ -8348,7 +8506,11 @@
         <v>72769</v>
       </c>
       <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>1781977009943</t>
+        </is>
+      </c>
       <c r="O52" t="n">
         <v>0</v>
       </c>
@@ -8369,7 +8531,11 @@
         <v>0</v>
       </c>
       <c r="V52" t="inlineStr"/>
-      <c r="W52" t="inlineStr"/>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5320/72073/32ce39ca-d5ae-499c-8117-a4df25d1ac9a.jpg</t>
+        </is>
+      </c>
       <c r="X52" t="n">
         <v>0</v>
       </c>
@@ -8497,7 +8663,11 @@
         <v>72770</v>
       </c>
       <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>1781976973878</t>
+        </is>
+      </c>
       <c r="O53" t="n">
         <v>0</v>
       </c>
@@ -8518,7 +8688,11 @@
         <v>0</v>
       </c>
       <c r="V53" t="inlineStr"/>
-      <c r="W53" t="inlineStr"/>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5320/72074/a7e9f42c-76c5-4e07-9e5d-4fef1c9084c2.jpg</t>
+        </is>
+      </c>
       <c r="X53" t="n">
         <v>0</v>
       </c>
@@ -8952,7 +9126,11 @@
         <v>72773</v>
       </c>
       <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>1781976760069</t>
+        </is>
+      </c>
       <c r="O56" t="n">
         <v>0</v>
       </c>
@@ -8973,7 +9151,11 @@
         <v>0</v>
       </c>
       <c r="V56" t="inlineStr"/>
-      <c r="W56" t="inlineStr"/>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5320/72077/2a634465-7213-4d7d-b2a0-c01dd558898c.jpg</t>
+        </is>
+      </c>
       <c r="X56" t="n">
         <v>0</v>
       </c>
@@ -9101,7 +9283,11 @@
         <v>72774</v>
       </c>
       <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>1781976895268</t>
+        </is>
+      </c>
       <c r="O57" t="n">
         <v>0</v>
       </c>
@@ -9122,7 +9308,11 @@
         <v>0</v>
       </c>
       <c r="V57" t="inlineStr"/>
-      <c r="W57" t="inlineStr"/>
+      <c r="W57" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5320/72078/1aef4a62-37d2-4dc8-a37d-4c155256568d.jpg</t>
+        </is>
+      </c>
       <c r="X57" t="n">
         <v>0</v>
       </c>
@@ -9407,7 +9597,11 @@
         <v>72776</v>
       </c>
       <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>1781976787558</t>
+        </is>
+      </c>
       <c r="O59" t="n">
         <v>0</v>
       </c>
@@ -9428,7 +9622,11 @@
         <v>0</v>
       </c>
       <c r="V59" t="inlineStr"/>
-      <c r="W59" t="inlineStr"/>
+      <c r="W59" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5320/72080/4fc33d99-a7d4-4de1-ada3-4b2bfd766083.jpg</t>
+        </is>
+      </c>
       <c r="X59" t="n">
         <v>0</v>
       </c>
@@ -9862,7 +10060,11 @@
         <v>154300</v>
       </c>
       <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr"/>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>1781976904577</t>
+        </is>
+      </c>
       <c r="O62" t="n">
         <v>0</v>
       </c>
@@ -9883,7 +10085,11 @@
         <v>0</v>
       </c>
       <c r="V62" t="inlineStr"/>
-      <c r="W62" t="inlineStr"/>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5320/649587/b45fbc5d-19b3-42bc-a371-ed180f83d40f.jpg</t>
+        </is>
+      </c>
       <c r="X62" t="n">
         <v>0</v>
       </c>
@@ -10011,7 +10217,11 @@
         <v>154301</v>
       </c>
       <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>1781977160840</t>
+        </is>
+      </c>
       <c r="O63" t="n">
         <v>0</v>
       </c>
@@ -10032,7 +10242,11 @@
         <v>0</v>
       </c>
       <c r="V63" t="inlineStr"/>
-      <c r="W63" t="inlineStr"/>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5320/649588/47f61f0d-1c98-42a2-a6bd-48dd47418273.jpg</t>
+        </is>
+      </c>
       <c r="X63" t="n">
         <v>0</v>
       </c>
@@ -10317,7 +10531,11 @@
         <v>154303</v>
       </c>
       <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>1781976902855</t>
+        </is>
+      </c>
       <c r="O65" t="n">
         <v>0</v>
       </c>
@@ -10338,7 +10556,11 @@
         <v>0</v>
       </c>
       <c r="V65" t="inlineStr"/>
-      <c r="W65" t="inlineStr"/>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5320/649590/d38d8aed-8ae0-4338-a620-bf7a0f4ae512.jpg</t>
+        </is>
+      </c>
       <c r="X65" t="n">
         <v>0</v>
       </c>
@@ -10466,7 +10688,11 @@
         <v>154304</v>
       </c>
       <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>1781976799614</t>
+        </is>
+      </c>
       <c r="O66" t="n">
         <v>0</v>
       </c>
@@ -10487,7 +10713,11 @@
         <v>0</v>
       </c>
       <c r="V66" t="inlineStr"/>
-      <c r="W66" t="inlineStr"/>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5320/649591/11ebeeeb-a7f0-4507-9130-05e51d8edfc8.jpg</t>
+        </is>
+      </c>
       <c r="X66" t="n">
         <v>0</v>
       </c>
@@ -10615,7 +10845,11 @@
         <v>154305</v>
       </c>
       <c r="M67" t="inlineStr"/>
-      <c r="N67" t="inlineStr"/>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>1781976975171</t>
+        </is>
+      </c>
       <c r="O67" t="n">
         <v>0</v>
       </c>
@@ -10636,7 +10870,11 @@
         <v>0</v>
       </c>
       <c r="V67" t="inlineStr"/>
-      <c r="W67" t="inlineStr"/>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5320/649592/5e3d533f-e739-4357-abd9-941b0bf4b5e6.jpg</t>
+        </is>
+      </c>
       <c r="X67" t="n">
         <v>0</v>
       </c>
@@ -10921,7 +11159,11 @@
         <v>154307</v>
       </c>
       <c r="M69" t="inlineStr"/>
-      <c r="N69" t="inlineStr"/>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>1781976912981</t>
+        </is>
+      </c>
       <c r="O69" t="n">
         <v>0</v>
       </c>
@@ -10942,7 +11184,11 @@
         <v>0</v>
       </c>
       <c r="V69" t="inlineStr"/>
-      <c r="W69" t="inlineStr"/>
+      <c r="W69" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5320/649594/0093dc8b-26cf-428d-a651-4d83c83f47a6.jpg</t>
+        </is>
+      </c>
       <c r="X69" t="n">
         <v>0</v>
       </c>
@@ -11070,7 +11316,11 @@
         <v>154308</v>
       </c>
       <c r="M70" t="inlineStr"/>
-      <c r="N70" t="inlineStr"/>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>1781976884239</t>
+        </is>
+      </c>
       <c r="O70" t="n">
         <v>0</v>
       </c>
@@ -11091,7 +11341,11 @@
         <v>0</v>
       </c>
       <c r="V70" t="inlineStr"/>
-      <c r="W70" t="inlineStr"/>
+      <c r="W70" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5320/649595/850e358d-30bc-4b10-b542-52b8d3cbd721.jpg</t>
+        </is>
+      </c>
       <c r="X70" t="n">
         <v>0</v>
       </c>
@@ -11219,7 +11473,11 @@
         <v>154309</v>
       </c>
       <c r="M71" t="inlineStr"/>
-      <c r="N71" t="inlineStr"/>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>1781976929176</t>
+        </is>
+      </c>
       <c r="O71" t="n">
         <v>0</v>
       </c>
@@ -11240,7 +11498,11 @@
         <v>0</v>
       </c>
       <c r="V71" t="inlineStr"/>
-      <c r="W71" t="inlineStr"/>
+      <c r="W71" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5320/649596/e42fdfda-91a3-4704-b57a-1b99d55fe96f.jpg</t>
+        </is>
+      </c>
       <c r="X71" t="n">
         <v>0</v>
       </c>
@@ -11525,7 +11787,11 @@
         <v>154311</v>
       </c>
       <c r="M73" t="inlineStr"/>
-      <c r="N73" t="inlineStr"/>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>1781977085167</t>
+        </is>
+      </c>
       <c r="O73" t="n">
         <v>0</v>
       </c>
@@ -11546,7 +11812,11 @@
         <v>0</v>
       </c>
       <c r="V73" t="inlineStr"/>
-      <c r="W73" t="inlineStr"/>
+      <c r="W73" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5320/649598/4d39134c-10d8-47e9-a1e1-9cfa67446092.jpg</t>
+        </is>
+      </c>
       <c r="X73" t="n">
         <v>0</v>
       </c>
@@ -11674,7 +11944,11 @@
         <v>154312</v>
       </c>
       <c r="M74" t="inlineStr"/>
-      <c r="N74" t="inlineStr"/>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>1781976940641</t>
+        </is>
+      </c>
       <c r="O74" t="n">
         <v>0</v>
       </c>
@@ -11695,7 +11969,11 @@
         <v>0</v>
       </c>
       <c r="V74" t="inlineStr"/>
-      <c r="W74" t="inlineStr"/>
+      <c r="W74" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5320/649599/2ff82a75-5864-4857-b0cb-8c72192a5d46.jpg</t>
+        </is>
+      </c>
       <c r="X74" t="n">
         <v>0</v>
       </c>
@@ -11823,7 +12101,11 @@
         <v>154313</v>
       </c>
       <c r="M75" t="inlineStr"/>
-      <c r="N75" t="inlineStr"/>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>1781976749086</t>
+        </is>
+      </c>
       <c r="O75" t="n">
         <v>0</v>
       </c>
@@ -11844,7 +12126,11 @@
         <v>0</v>
       </c>
       <c r="V75" t="inlineStr"/>
-      <c r="W75" t="inlineStr"/>
+      <c r="W75" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5320/649600/6d250949-9ae0-4fa5-a1da-b8e45a7c68bf.jpg</t>
+        </is>
+      </c>
       <c r="X75" t="n">
         <v>0</v>
       </c>
@@ -12128,29 +12414,43 @@
       <c r="L77" t="n">
         <v>72780</v>
       </c>
-      <c r="M77" t="inlineStr"/>
-      <c r="N77" t="inlineStr"/>
+      <c r="M77" t="n">
+        <v>1781976826191</v>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>1781976825590</t>
+        </is>
+      </c>
       <c r="O77" t="n">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="P77" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="Q77" t="n">
         <v>0</v>
       </c>
-      <c r="R77" t="inlineStr"/>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>6a36cef9370583337b6e7091</t>
+        </is>
+      </c>
       <c r="S77" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="T77" t="n">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="U77" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="V77" t="inlineStr"/>
-      <c r="W77" t="inlineStr"/>
+      <c r="W77" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/72084/80b9f651-9b8c-4e3b-a2d3-885e0fadc0ce.jpg</t>
+        </is>
+      </c>
       <c r="X77" t="n">
         <v>0</v>
       </c>
@@ -12167,7 +12467,7 @@
         <v>0</v>
       </c>
       <c r="AC77" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="AD77" t="n">
         <v>0</v>
@@ -12185,7 +12485,7 @@
         <v>0</v>
       </c>
       <c r="AI77" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AJ77" t="n">
         <v>0</v>
@@ -13345,7 +13645,11 @@
         <v>72788</v>
       </c>
       <c r="M85" t="inlineStr"/>
-      <c r="N85" t="inlineStr"/>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>1781976808001</t>
+        </is>
+      </c>
       <c r="O85" t="n">
         <v>0</v>
       </c>
@@ -13366,7 +13670,11 @@
         <v>0</v>
       </c>
       <c r="V85" t="inlineStr"/>
-      <c r="W85" t="inlineStr"/>
+      <c r="W85" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/72092/db0a491f-f559-49bd-b17f-248037832ca9.jpg</t>
+        </is>
+      </c>
       <c r="X85" t="n">
         <v>0</v>
       </c>
@@ -13643,7 +13951,11 @@
         <v>72790</v>
       </c>
       <c r="M87" t="inlineStr"/>
-      <c r="N87" t="inlineStr"/>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>1781976801411</t>
+        </is>
+      </c>
       <c r="O87" t="n">
         <v>0</v>
       </c>
@@ -13664,7 +13976,11 @@
         <v>0</v>
       </c>
       <c r="V87" t="inlineStr"/>
-      <c r="W87" t="inlineStr"/>
+      <c r="W87" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/72094/ec06b031-2321-49c1-899d-4bacabb88baa.jpg</t>
+        </is>
+      </c>
       <c r="X87" t="n">
         <v>0</v>
       </c>
@@ -14426,7 +14742,11 @@
         <v>72795</v>
       </c>
       <c r="M92" t="inlineStr"/>
-      <c r="N92" t="inlineStr"/>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>1781977012987</t>
+        </is>
+      </c>
       <c r="O92" t="n">
         <v>0</v>
       </c>
@@ -14447,7 +14767,11 @@
         <v>0</v>
       </c>
       <c r="V92" t="inlineStr"/>
-      <c r="W92" t="inlineStr"/>
+      <c r="W92" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/72099/016589e6-743c-4bd0-92c2-929326e5ccf2.jpg</t>
+        </is>
+      </c>
       <c r="X92" t="n">
         <v>0</v>
       </c>
@@ -15187,7 +15511,11 @@
         <v>154317</v>
       </c>
       <c r="M97" t="inlineStr"/>
-      <c r="N97" t="inlineStr"/>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>1781976898756</t>
+        </is>
+      </c>
       <c r="O97" t="n">
         <v>0</v>
       </c>
@@ -15208,7 +15536,11 @@
         <v>0</v>
       </c>
       <c r="V97" t="inlineStr"/>
-      <c r="W97" t="inlineStr"/>
+      <c r="W97" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/649606/82491a2d-0f3d-4d21-8e2b-4545c926cd92.jpg</t>
+        </is>
+      </c>
       <c r="X97" t="n">
         <v>0</v>
       </c>
@@ -15336,7 +15668,11 @@
         <v>154318</v>
       </c>
       <c r="M98" t="inlineStr"/>
-      <c r="N98" t="inlineStr"/>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>1781977035978</t>
+        </is>
+      </c>
       <c r="O98" t="n">
         <v>0</v>
       </c>
@@ -15357,7 +15693,11 @@
         <v>0</v>
       </c>
       <c r="V98" t="inlineStr"/>
-      <c r="W98" t="inlineStr"/>
+      <c r="W98" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/649607/1538d91d-3f4b-4e0d-8cbf-e9e5ee67944d.jpg</t>
+        </is>
+      </c>
       <c r="X98" t="n">
         <v>0</v>
       </c>
@@ -16725,7 +17065,11 @@
         <v>154327</v>
       </c>
       <c r="M107" t="inlineStr"/>
-      <c r="N107" t="inlineStr"/>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>1781976939375</t>
+        </is>
+      </c>
       <c r="O107" t="n">
         <v>0</v>
       </c>
@@ -16746,7 +17090,11 @@
         <v>0</v>
       </c>
       <c r="V107" t="inlineStr"/>
-      <c r="W107" t="inlineStr"/>
+      <c r="W107" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/649616/1247d470-53bf-419a-9c44-bea4ca5b6eaf.jpg</t>
+        </is>
+      </c>
       <c r="X107" t="n">
         <v>0</v>
       </c>
@@ -16874,7 +17222,11 @@
         <v>154328</v>
       </c>
       <c r="M108" t="inlineStr"/>
-      <c r="N108" t="inlineStr"/>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>1781976765857</t>
+        </is>
+      </c>
       <c r="O108" t="n">
         <v>0</v>
       </c>
@@ -16895,7 +17247,11 @@
         <v>0</v>
       </c>
       <c r="V108" t="inlineStr"/>
-      <c r="W108" t="inlineStr"/>
+      <c r="W108" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/649617/868af142-1ece-49a1-937a-7e3db1ebdea6.jpg</t>
+        </is>
+      </c>
       <c r="X108" t="n">
         <v>0</v>
       </c>
@@ -17329,7 +17685,11 @@
         <v>154331</v>
       </c>
       <c r="M111" t="inlineStr"/>
-      <c r="N111" t="inlineStr"/>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>1781976792840</t>
+        </is>
+      </c>
       <c r="O111" t="n">
         <v>0</v>
       </c>
@@ -17350,7 +17710,11 @@
         <v>0</v>
       </c>
       <c r="V111" t="inlineStr"/>
-      <c r="W111" t="inlineStr"/>
+      <c r="W111" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/649620/3269b8ca-479f-44b0-bedb-86ce76546578.jpg</t>
+        </is>
+      </c>
       <c r="X111" t="n">
         <v>0</v>
       </c>
@@ -17784,7 +18148,11 @@
         <v>154334</v>
       </c>
       <c r="M114" t="inlineStr"/>
-      <c r="N114" t="inlineStr"/>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>1781977103011</t>
+        </is>
+      </c>
       <c r="O114" t="n">
         <v>0</v>
       </c>
@@ -17805,7 +18173,11 @@
         <v>0</v>
       </c>
       <c r="V114" t="inlineStr"/>
-      <c r="W114" t="inlineStr"/>
+      <c r="W114" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/649623/dadbf14d-4d31-405b-99aa-05514292e85a.jpg</t>
+        </is>
+      </c>
       <c r="X114" t="n">
         <v>0</v>
       </c>
@@ -18090,7 +18462,11 @@
         <v>154336</v>
       </c>
       <c r="M116" t="inlineStr"/>
-      <c r="N116" t="inlineStr"/>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>1781976856628</t>
+        </is>
+      </c>
       <c r="O116" t="n">
         <v>0</v>
       </c>
@@ -18111,7 +18487,11 @@
         <v>0</v>
       </c>
       <c r="V116" t="inlineStr"/>
-      <c r="W116" t="inlineStr"/>
+      <c r="W116" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/649625/e08a9e5f-9424-47e7-a31b-01007dba954b.jpg</t>
+        </is>
+      </c>
       <c r="X116" t="n">
         <v>0</v>
       </c>
@@ -18396,7 +18776,11 @@
         <v>154338</v>
       </c>
       <c r="M118" t="inlineStr"/>
-      <c r="N118" t="inlineStr"/>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>1781976604167</t>
+        </is>
+      </c>
       <c r="O118" t="n">
         <v>0</v>
       </c>
@@ -18417,7 +18801,11 @@
         <v>0</v>
       </c>
       <c r="V118" t="inlineStr"/>
-      <c r="W118" t="inlineStr"/>
+      <c r="W118" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/649627/4c1b9cd6-31e9-4a09-941c-6d6460ed05ce.jpg</t>
+        </is>
+      </c>
       <c r="X118" t="n">
         <v>0</v>
       </c>
@@ -18851,7 +19239,11 @@
         <v>154341</v>
       </c>
       <c r="M121" t="inlineStr"/>
-      <c r="N121" t="inlineStr"/>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>1781976800351</t>
+        </is>
+      </c>
       <c r="O121" t="n">
         <v>0</v>
       </c>
@@ -18872,7 +19264,11 @@
         <v>0</v>
       </c>
       <c r="V121" t="inlineStr"/>
-      <c r="W121" t="inlineStr"/>
+      <c r="W121" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5321/649630/05971cd9-bfea-49bf-8a4b-21143ff2c470.jpg</t>
+        </is>
+      </c>
       <c r="X121" t="n">
         <v>0</v>
       </c>
@@ -19320,7 +19716,11 @@
         <v>72798</v>
       </c>
       <c r="M124" t="inlineStr"/>
-      <c r="N124" t="inlineStr"/>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>1781976753311</t>
+        </is>
+      </c>
       <c r="O124" t="n">
         <v>0</v>
       </c>
@@ -19341,7 +19741,11 @@
         <v>0</v>
       </c>
       <c r="V124" t="inlineStr"/>
-      <c r="W124" t="inlineStr"/>
+      <c r="W124" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/72102/40ab74b3-e839-4f85-9dab-ad170e54af91.jpg</t>
+        </is>
+      </c>
       <c r="X124" t="n">
         <v>0</v>
       </c>
@@ -19469,7 +19873,11 @@
         <v>72799</v>
       </c>
       <c r="M125" t="inlineStr"/>
-      <c r="N125" t="inlineStr"/>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>1781977072233</t>
+        </is>
+      </c>
       <c r="O125" t="n">
         <v>0</v>
       </c>
@@ -19490,7 +19898,11 @@
         <v>0</v>
       </c>
       <c r="V125" t="inlineStr"/>
-      <c r="W125" t="inlineStr"/>
+      <c r="W125" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/72103/62d5ac82-06b5-45a7-bf94-1c06eddeaef3.jpg</t>
+        </is>
+      </c>
       <c r="X125" t="n">
         <v>0</v>
       </c>
@@ -19767,7 +20179,11 @@
         <v>72801</v>
       </c>
       <c r="M127" t="inlineStr"/>
-      <c r="N127" t="inlineStr"/>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>1781977028685</t>
+        </is>
+      </c>
       <c r="O127" t="n">
         <v>0</v>
       </c>
@@ -19788,7 +20204,11 @@
         <v>0</v>
       </c>
       <c r="V127" t="inlineStr"/>
-      <c r="W127" t="inlineStr"/>
+      <c r="W127" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/72105/f81881b5-119b-458d-843a-2b19327d1f59.jpg</t>
+        </is>
+      </c>
       <c r="X127" t="n">
         <v>0</v>
       </c>
@@ -20073,7 +20493,11 @@
         <v>72803</v>
       </c>
       <c r="M129" t="inlineStr"/>
-      <c r="N129" t="inlineStr"/>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>1781976897688</t>
+        </is>
+      </c>
       <c r="O129" t="n">
         <v>0</v>
       </c>
@@ -20094,7 +20518,11 @@
         <v>0</v>
       </c>
       <c r="V129" t="inlineStr"/>
-      <c r="W129" t="inlineStr"/>
+      <c r="W129" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/72107/f4767b63-1f05-4272-bd81-0176f6550e9d.jpg</t>
+        </is>
+      </c>
       <c r="X129" t="n">
         <v>0</v>
       </c>
@@ -20222,7 +20650,11 @@
         <v>72804</v>
       </c>
       <c r="M130" t="inlineStr"/>
-      <c r="N130" t="inlineStr"/>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>1781976757459</t>
+        </is>
+      </c>
       <c r="O130" t="n">
         <v>0</v>
       </c>
@@ -20243,7 +20675,11 @@
         <v>0</v>
       </c>
       <c r="V130" t="inlineStr"/>
-      <c r="W130" t="inlineStr"/>
+      <c r="W130" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/72108/7e70c4f0-15a8-40c6-a3ba-1382f65fb4ea.jpg</t>
+        </is>
+      </c>
       <c r="X130" t="n">
         <v>0</v>
       </c>
@@ -20371,7 +20807,11 @@
         <v>72805</v>
       </c>
       <c r="M131" t="inlineStr"/>
-      <c r="N131" t="inlineStr"/>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t>1781976878316</t>
+        </is>
+      </c>
       <c r="O131" t="n">
         <v>0</v>
       </c>
@@ -20392,7 +20832,11 @@
         <v>0</v>
       </c>
       <c r="V131" t="inlineStr"/>
-      <c r="W131" t="inlineStr"/>
+      <c r="W131" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/72109/98a815c8-f888-40d9-823d-943b79e22682.jpg</t>
+        </is>
+      </c>
       <c r="X131" t="n">
         <v>0</v>
       </c>
@@ -20520,7 +20964,11 @@
         <v>154343</v>
       </c>
       <c r="M132" t="inlineStr"/>
-      <c r="N132" t="inlineStr"/>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t>1781977091793</t>
+        </is>
+      </c>
       <c r="O132" t="n">
         <v>0</v>
       </c>
@@ -20541,7 +20989,11 @@
         <v>0</v>
       </c>
       <c r="V132" t="inlineStr"/>
-      <c r="W132" t="inlineStr"/>
+      <c r="W132" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/649632/ad33cec4-309d-47c5-bc85-c54f3dd3ee52.jpg</t>
+        </is>
+      </c>
       <c r="X132" t="n">
         <v>0</v>
       </c>
@@ -20669,7 +21121,11 @@
         <v>154344</v>
       </c>
       <c r="M133" t="inlineStr"/>
-      <c r="N133" t="inlineStr"/>
+      <c r="N133" t="inlineStr">
+        <is>
+          <t>1781976811468</t>
+        </is>
+      </c>
       <c r="O133" t="n">
         <v>0</v>
       </c>
@@ -20690,7 +21146,11 @@
         <v>0</v>
       </c>
       <c r="V133" t="inlineStr"/>
-      <c r="W133" t="inlineStr"/>
+      <c r="W133" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/649633/83d2ee5c-a8aa-412d-8af8-b174eba8c621.jpg</t>
+        </is>
+      </c>
       <c r="X133" t="n">
         <v>0</v>
       </c>
@@ -20818,7 +21278,11 @@
         <v>154345</v>
       </c>
       <c r="M134" t="inlineStr"/>
-      <c r="N134" t="inlineStr"/>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>1781976813220</t>
+        </is>
+      </c>
       <c r="O134" t="n">
         <v>0</v>
       </c>
@@ -20839,7 +21303,11 @@
         <v>0</v>
       </c>
       <c r="V134" t="inlineStr"/>
-      <c r="W134" t="inlineStr"/>
+      <c r="W134" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/649634/5eda984a-d04a-48f2-b3f0-8ba74548dcbc.jpg</t>
+        </is>
+      </c>
       <c r="X134" t="n">
         <v>0</v>
       </c>
@@ -21124,7 +21592,11 @@
         <v>154347</v>
       </c>
       <c r="M136" t="inlineStr"/>
-      <c r="N136" t="inlineStr"/>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>1781977084016</t>
+        </is>
+      </c>
       <c r="O136" t="n">
         <v>0</v>
       </c>
@@ -21145,7 +21617,11 @@
         <v>0</v>
       </c>
       <c r="V136" t="inlineStr"/>
-      <c r="W136" t="inlineStr"/>
+      <c r="W136" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/649636/66341247-9bca-4315-b48a-8ac2e4bad1f6.jpg</t>
+        </is>
+      </c>
       <c r="X136" t="n">
         <v>0</v>
       </c>
@@ -21587,7 +22063,11 @@
         <v>154350</v>
       </c>
       <c r="M139" t="inlineStr"/>
-      <c r="N139" t="inlineStr"/>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>1781977141257</t>
+        </is>
+      </c>
       <c r="O139" t="n">
         <v>0</v>
       </c>
@@ -21608,7 +22088,11 @@
         <v>0</v>
       </c>
       <c r="V139" t="inlineStr"/>
-      <c r="W139" t="inlineStr"/>
+      <c r="W139" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/649639/db060d47-ace5-43e4-a74c-87a92736c200.jpg</t>
+        </is>
+      </c>
       <c r="X139" t="n">
         <v>0</v>
       </c>
@@ -21736,7 +22220,11 @@
         <v>154351</v>
       </c>
       <c r="M140" t="inlineStr"/>
-      <c r="N140" t="inlineStr"/>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>1781976918004</t>
+        </is>
+      </c>
       <c r="O140" t="n">
         <v>0</v>
       </c>
@@ -21757,7 +22245,11 @@
         <v>0</v>
       </c>
       <c r="V140" t="inlineStr"/>
-      <c r="W140" t="inlineStr"/>
+      <c r="W140" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/649640/94b0a329-65fe-42a3-af30-cce5ecbfdec6.jpg</t>
+        </is>
+      </c>
       <c r="X140" t="n">
         <v>0</v>
       </c>
@@ -21885,7 +22377,11 @@
         <v>154352</v>
       </c>
       <c r="M141" t="inlineStr"/>
-      <c r="N141" t="inlineStr"/>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>1781976799738</t>
+        </is>
+      </c>
       <c r="O141" t="n">
         <v>0</v>
       </c>
@@ -21906,7 +22402,11 @@
         <v>0</v>
       </c>
       <c r="V141" t="inlineStr"/>
-      <c r="W141" t="inlineStr"/>
+      <c r="W141" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/649641/e6e9a162-ee13-4ba0-8d75-756a5f904523.jpg</t>
+        </is>
+      </c>
       <c r="X141" t="n">
         <v>0</v>
       </c>
@@ -22034,7 +22534,11 @@
         <v>154353</v>
       </c>
       <c r="M142" t="inlineStr"/>
-      <c r="N142" t="inlineStr"/>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>1781976776940</t>
+        </is>
+      </c>
       <c r="O142" t="n">
         <v>0</v>
       </c>
@@ -22055,7 +22559,11 @@
         <v>0</v>
       </c>
       <c r="V142" t="inlineStr"/>
-      <c r="W142" t="inlineStr"/>
+      <c r="W142" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/649642/387b88fd-2c13-4f36-a8d6-916eb22af60a.jpg</t>
+        </is>
+      </c>
       <c r="X142" t="n">
         <v>0</v>
       </c>
@@ -22183,7 +22691,11 @@
         <v>154354</v>
       </c>
       <c r="M143" t="inlineStr"/>
-      <c r="N143" t="inlineStr"/>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>1781976873452</t>
+        </is>
+      </c>
       <c r="O143" t="n">
         <v>0</v>
       </c>
@@ -22204,7 +22716,11 @@
         <v>0</v>
       </c>
       <c r="V143" t="inlineStr"/>
-      <c r="W143" t="inlineStr"/>
+      <c r="W143" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/649643/317d612c-b56f-4238-b272-987c5a701ce4.jpg</t>
+        </is>
+      </c>
       <c r="X143" t="n">
         <v>0</v>
       </c>
@@ -22332,7 +22848,11 @@
         <v>154355</v>
       </c>
       <c r="M144" t="inlineStr"/>
-      <c r="N144" t="inlineStr"/>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>1781977000020</t>
+        </is>
+      </c>
       <c r="O144" t="n">
         <v>0</v>
       </c>
@@ -22353,7 +22873,11 @@
         <v>0</v>
       </c>
       <c r="V144" t="inlineStr"/>
-      <c r="W144" t="inlineStr"/>
+      <c r="W144" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/649644/18403d7b-061f-4fa8-a587-82c1ce0430d7.jpg</t>
+        </is>
+      </c>
       <c r="X144" t="n">
         <v>0</v>
       </c>
@@ -22481,7 +23005,11 @@
         <v>154356</v>
       </c>
       <c r="M145" t="inlineStr"/>
-      <c r="N145" t="inlineStr"/>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>1781976898853</t>
+        </is>
+      </c>
       <c r="O145" t="n">
         <v>0</v>
       </c>
@@ -22502,7 +23030,11 @@
         <v>0</v>
       </c>
       <c r="V145" t="inlineStr"/>
-      <c r="W145" t="inlineStr"/>
+      <c r="W145" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/649645/c7bfaeb8-5721-4fe5-b42f-e5872d1afb38.jpg</t>
+        </is>
+      </c>
       <c r="X145" t="n">
         <v>0</v>
       </c>
@@ -22630,7 +23162,11 @@
         <v>154357</v>
       </c>
       <c r="M146" t="inlineStr"/>
-      <c r="N146" t="inlineStr"/>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>1781976887946</t>
+        </is>
+      </c>
       <c r="O146" t="n">
         <v>0</v>
       </c>
@@ -22651,7 +23187,11 @@
         <v>0</v>
       </c>
       <c r="V146" t="inlineStr"/>
-      <c r="W146" t="inlineStr"/>
+      <c r="W146" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/649646/373f5c76-a9ce-4dc4-a759-923c41b9913b.jpg</t>
+        </is>
+      </c>
       <c r="X146" t="n">
         <v>0</v>
       </c>
@@ -22779,7 +23319,11 @@
         <v>154358</v>
       </c>
       <c r="M147" t="inlineStr"/>
-      <c r="N147" t="inlineStr"/>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>1781976903989</t>
+        </is>
+      </c>
       <c r="O147" t="n">
         <v>0</v>
       </c>
@@ -22800,7 +23344,11 @@
         <v>0</v>
       </c>
       <c r="V147" t="inlineStr"/>
-      <c r="W147" t="inlineStr"/>
+      <c r="W147" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/649647/c0286499-10c5-4a46-9990-c6b353c76c82.jpg</t>
+        </is>
+      </c>
       <c r="X147" t="n">
         <v>0</v>
       </c>
@@ -23085,7 +23633,11 @@
         <v>154360</v>
       </c>
       <c r="M149" t="inlineStr"/>
-      <c r="N149" t="inlineStr"/>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>1781976749631</t>
+        </is>
+      </c>
       <c r="O149" t="n">
         <v>0</v>
       </c>
@@ -23106,7 +23658,11 @@
         <v>0</v>
       </c>
       <c r="V149" t="inlineStr"/>
-      <c r="W149" t="inlineStr"/>
+      <c r="W149" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5322/649649/419eb691-04f5-4cd1-b49d-0c1d818481a4.jpg</t>
+        </is>
+      </c>
       <c r="X149" t="n">
         <v>0</v>
       </c>
@@ -23711,7 +24267,11 @@
         <v>72808</v>
       </c>
       <c r="M153" t="inlineStr"/>
-      <c r="N153" t="inlineStr"/>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>1781976793577</t>
+        </is>
+      </c>
       <c r="O153" t="n">
         <v>0</v>
       </c>
@@ -23732,7 +24292,11 @@
         <v>0</v>
       </c>
       <c r="V153" t="inlineStr"/>
-      <c r="W153" t="inlineStr"/>
+      <c r="W153" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5323/72112/1c46c209-400e-42d0-8fc3-b8897559840d.jpg</t>
+        </is>
+      </c>
       <c r="X153" t="n">
         <v>0</v>
       </c>
@@ -24017,7 +24581,11 @@
         <v>72810</v>
       </c>
       <c r="M155" t="inlineStr"/>
-      <c r="N155" t="inlineStr"/>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>1781976916801</t>
+        </is>
+      </c>
       <c r="O155" t="n">
         <v>0</v>
       </c>
@@ -24038,7 +24606,11 @@
         <v>0</v>
       </c>
       <c r="V155" t="inlineStr"/>
-      <c r="W155" t="inlineStr"/>
+      <c r="W155" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5323/72114/9f7b9cd7-47e9-4e7a-bbcf-2671dc141d00.jpg</t>
+        </is>
+      </c>
       <c r="X155" t="n">
         <v>0</v>
       </c>
@@ -24323,7 +24895,11 @@
         <v>72812</v>
       </c>
       <c r="M157" t="inlineStr"/>
-      <c r="N157" t="inlineStr"/>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>1781976825354</t>
+        </is>
+      </c>
       <c r="O157" t="n">
         <v>0</v>
       </c>
@@ -24344,7 +24920,11 @@
         <v>0</v>
       </c>
       <c r="V157" t="inlineStr"/>
-      <c r="W157" t="inlineStr"/>
+      <c r="W157" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5323/72116/327d5ebd-13f6-44d2-9d7b-67b4811065c0.jpg</t>
+        </is>
+      </c>
       <c r="X157" t="n">
         <v>0</v>
       </c>
@@ -24786,7 +25366,11 @@
         <v>154364</v>
       </c>
       <c r="M160" t="inlineStr"/>
-      <c r="N160" t="inlineStr"/>
+      <c r="N160" t="inlineStr">
+        <is>
+          <t>1781977143749</t>
+        </is>
+      </c>
       <c r="O160" t="n">
         <v>0</v>
       </c>
@@ -24807,7 +25391,11 @@
         <v>0</v>
       </c>
       <c r="V160" t="inlineStr"/>
-      <c r="W160" t="inlineStr"/>
+      <c r="W160" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5323/649653/32ede705-a440-47ed-92e5-efeb6efddaa6.jpg</t>
+        </is>
+      </c>
       <c r="X160" t="n">
         <v>0</v>
       </c>
@@ -24935,7 +25523,11 @@
         <v>154365</v>
       </c>
       <c r="M161" t="inlineStr"/>
-      <c r="N161" t="inlineStr"/>
+      <c r="N161" t="inlineStr">
+        <is>
+          <t>1781976944335</t>
+        </is>
+      </c>
       <c r="O161" t="n">
         <v>0</v>
       </c>
@@ -24956,7 +25548,11 @@
         <v>0</v>
       </c>
       <c r="V161" t="inlineStr"/>
-      <c r="W161" t="inlineStr"/>
+      <c r="W161" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5323/649654/235ab69c-bd5a-4f12-9c62-5c50b005314f.jpg</t>
+        </is>
+      </c>
       <c r="X161" t="n">
         <v>0</v>
       </c>
@@ -25233,7 +25829,11 @@
         <v>72814</v>
       </c>
       <c r="M163" t="inlineStr"/>
-      <c r="N163" t="inlineStr"/>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>1781976761622</t>
+        </is>
+      </c>
       <c r="O163" t="n">
         <v>0</v>
       </c>
@@ -25254,7 +25854,11 @@
         <v>0</v>
       </c>
       <c r="V163" t="inlineStr"/>
-      <c r="W163" t="inlineStr"/>
+      <c r="W163" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5324/72118/978d9f15-5869-4cb8-be4e-ff7c3c3651a1.jpg</t>
+        </is>
+      </c>
       <c r="X163" t="n">
         <v>0</v>
       </c>
@@ -25539,7 +26143,11 @@
         <v>72816</v>
       </c>
       <c r="M165" t="inlineStr"/>
-      <c r="N165" t="inlineStr"/>
+      <c r="N165" t="inlineStr">
+        <is>
+          <t>1781976926205</t>
+        </is>
+      </c>
       <c r="O165" t="n">
         <v>0</v>
       </c>
@@ -25560,7 +26168,11 @@
         <v>0</v>
       </c>
       <c r="V165" t="inlineStr"/>
-      <c r="W165" t="inlineStr"/>
+      <c r="W165" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5324/72120/ceabef35-cc65-4eb1-9ee7-34891f70721d.jpg</t>
+        </is>
+      </c>
       <c r="X165" t="n">
         <v>0</v>
       </c>
@@ -25688,7 +26300,11 @@
         <v>72817</v>
       </c>
       <c r="M166" t="inlineStr"/>
-      <c r="N166" t="inlineStr"/>
+      <c r="N166" t="inlineStr">
+        <is>
+          <t>1781976815150</t>
+        </is>
+      </c>
       <c r="O166" t="n">
         <v>0</v>
       </c>
@@ -25709,7 +26325,11 @@
         <v>0</v>
       </c>
       <c r="V166" t="inlineStr"/>
-      <c r="W166" t="inlineStr"/>
+      <c r="W166" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5324/72121/5319c255-72ed-49c8-8a2f-299e19051bf0.jpg</t>
+        </is>
+      </c>
       <c r="X166" t="n">
         <v>0</v>
       </c>
@@ -25837,7 +26457,11 @@
         <v>72818</v>
       </c>
       <c r="M167" t="inlineStr"/>
-      <c r="N167" t="inlineStr"/>
+      <c r="N167" t="inlineStr">
+        <is>
+          <t>1781976808039</t>
+        </is>
+      </c>
       <c r="O167" t="n">
         <v>0</v>
       </c>
@@ -25858,7 +26482,11 @@
         <v>0</v>
       </c>
       <c r="V167" t="inlineStr"/>
-      <c r="W167" t="inlineStr"/>
+      <c r="W167" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5324/72122/55e6a6e5-7344-4fc0-8171-d95efda89c84.jpg</t>
+        </is>
+      </c>
       <c r="X167" t="n">
         <v>0</v>
       </c>
@@ -25986,7 +26614,11 @@
         <v>72819</v>
       </c>
       <c r="M168" t="inlineStr"/>
-      <c r="N168" t="inlineStr"/>
+      <c r="N168" t="inlineStr">
+        <is>
+          <t>1781976856002</t>
+        </is>
+      </c>
       <c r="O168" t="n">
         <v>0</v>
       </c>
@@ -26007,7 +26639,11 @@
         <v>0</v>
       </c>
       <c r="V168" t="inlineStr"/>
-      <c r="W168" t="inlineStr"/>
+      <c r="W168" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5324/72123/c79ec65a-3bb4-4bed-81ec-f1a7b819ea10.jpg</t>
+        </is>
+      </c>
       <c r="X168" t="n">
         <v>0</v>
       </c>
@@ -26135,7 +26771,11 @@
         <v>72820</v>
       </c>
       <c r="M169" t="inlineStr"/>
-      <c r="N169" t="inlineStr"/>
+      <c r="N169" t="inlineStr">
+        <is>
+          <t>1781976975739</t>
+        </is>
+      </c>
       <c r="O169" t="n">
         <v>0</v>
       </c>
@@ -26156,7 +26796,11 @@
         <v>0</v>
       </c>
       <c r="V169" t="inlineStr"/>
-      <c r="W169" t="inlineStr"/>
+      <c r="W169" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5324/72124/95e219d1-2b36-4425-8f50-829c1516bd87.jpg</t>
+        </is>
+      </c>
       <c r="X169" t="n">
         <v>0</v>
       </c>
@@ -26284,7 +26928,11 @@
         <v>72821</v>
       </c>
       <c r="M170" t="inlineStr"/>
-      <c r="N170" t="inlineStr"/>
+      <c r="N170" t="inlineStr">
+        <is>
+          <t>1781976826852</t>
+        </is>
+      </c>
       <c r="O170" t="n">
         <v>0</v>
       </c>
@@ -26305,7 +26953,11 @@
         <v>0</v>
       </c>
       <c r="V170" t="inlineStr"/>
-      <c r="W170" t="inlineStr"/>
+      <c r="W170" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5324/72125/60e35c33-2c45-4d5c-8f4c-56e264f065d2.jpg</t>
+        </is>
+      </c>
       <c r="X170" t="n">
         <v>0</v>
       </c>
@@ -26433,7 +27085,11 @@
         <v>154366</v>
       </c>
       <c r="M171" t="inlineStr"/>
-      <c r="N171" t="inlineStr"/>
+      <c r="N171" t="inlineStr">
+        <is>
+          <t>1781976775802</t>
+        </is>
+      </c>
       <c r="O171" t="n">
         <v>0</v>
       </c>
@@ -26454,7 +27110,11 @@
         <v>0</v>
       </c>
       <c r="V171" t="inlineStr"/>
-      <c r="W171" t="inlineStr"/>
+      <c r="W171" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5324/649655/740c1e43-0b29-4878-b837-aa30f84a1063.jpg</t>
+        </is>
+      </c>
       <c r="X171" t="n">
         <v>0</v>
       </c>
@@ -27053,7 +27713,11 @@
         <v>154370</v>
       </c>
       <c r="M175" t="inlineStr"/>
-      <c r="N175" t="inlineStr"/>
+      <c r="N175" t="inlineStr">
+        <is>
+          <t>1781977008723</t>
+        </is>
+      </c>
       <c r="O175" t="n">
         <v>0</v>
       </c>
@@ -27074,7 +27738,11 @@
         <v>0</v>
       </c>
       <c r="V175" t="inlineStr"/>
-      <c r="W175" t="inlineStr"/>
+      <c r="W175" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5324/649659/5f7adc8c-f9bb-4501-8d3e-3004d625c186.jpg</t>
+        </is>
+      </c>
       <c r="X175" t="n">
         <v>0</v>
       </c>
@@ -27359,7 +28027,11 @@
         <v>154372</v>
       </c>
       <c r="M177" t="inlineStr"/>
-      <c r="N177" t="inlineStr"/>
+      <c r="N177" t="inlineStr">
+        <is>
+          <t>1781976806551</t>
+        </is>
+      </c>
       <c r="O177" t="n">
         <v>0</v>
       </c>
@@ -27380,7 +28052,11 @@
         <v>0</v>
       </c>
       <c r="V177" t="inlineStr"/>
-      <c r="W177" t="inlineStr"/>
+      <c r="W177" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5324/675488/5b87fca6-3889-420b-ab9b-ca42b8b1be59.jpg</t>
+        </is>
+      </c>
       <c r="X177" t="n">
         <v>0</v>
       </c>
@@ -27508,7 +28184,11 @@
         <v>72822</v>
       </c>
       <c r="M178" t="inlineStr"/>
-      <c r="N178" t="inlineStr"/>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>1781976920430</t>
+        </is>
+      </c>
       <c r="O178" t="n">
         <v>0</v>
       </c>
@@ -27529,7 +28209,11 @@
         <v>0</v>
       </c>
       <c r="V178" t="inlineStr"/>
-      <c r="W178" t="inlineStr"/>
+      <c r="W178" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5325/72126/00753055-b555-49a1-bcc5-9a10fcc259e9.jpg</t>
+        </is>
+      </c>
       <c r="X178" t="n">
         <v>0</v>
       </c>
@@ -27657,7 +28341,11 @@
         <v>72823</v>
       </c>
       <c r="M179" t="inlineStr"/>
-      <c r="N179" t="inlineStr"/>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>1781977087206</t>
+        </is>
+      </c>
       <c r="O179" t="n">
         <v>0</v>
       </c>
@@ -27678,7 +28366,11 @@
         <v>0</v>
       </c>
       <c r="V179" t="inlineStr"/>
-      <c r="W179" t="inlineStr"/>
+      <c r="W179" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5325/72127/3828d445-8d2b-40d3-80e1-9e398a874878.jpg</t>
+        </is>
+      </c>
       <c r="X179" t="n">
         <v>0</v>
       </c>
@@ -27806,7 +28498,11 @@
         <v>72824</v>
       </c>
       <c r="M180" t="inlineStr"/>
-      <c r="N180" t="inlineStr"/>
+      <c r="N180" t="inlineStr">
+        <is>
+          <t>1781977027399</t>
+        </is>
+      </c>
       <c r="O180" t="n">
         <v>0</v>
       </c>
@@ -27827,7 +28523,11 @@
         <v>0</v>
       </c>
       <c r="V180" t="inlineStr"/>
-      <c r="W180" t="inlineStr"/>
+      <c r="W180" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5325/72128/e5d63854-e59c-4730-bd60-a111d771280b.jpg</t>
+        </is>
+      </c>
       <c r="X180" t="n">
         <v>0</v>
       </c>
@@ -28583,7 +29283,11 @@
         <v>72829</v>
       </c>
       <c r="M185" t="inlineStr"/>
-      <c r="N185" t="inlineStr"/>
+      <c r="N185" t="inlineStr">
+        <is>
+          <t>1781976807397</t>
+        </is>
+      </c>
       <c r="O185" t="n">
         <v>0</v>
       </c>
@@ -28604,7 +29308,11 @@
         <v>0</v>
       </c>
       <c r="V185" t="inlineStr"/>
-      <c r="W185" t="inlineStr"/>
+      <c r="W185" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5325/72133/9718493c-05ff-45d9-9585-f87041450055.jpg</t>
+        </is>
+      </c>
       <c r="X185" t="n">
         <v>0</v>
       </c>
@@ -28732,7 +29440,11 @@
         <v>154373</v>
       </c>
       <c r="M186" t="inlineStr"/>
-      <c r="N186" t="inlineStr"/>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>1781976858966</t>
+        </is>
+      </c>
       <c r="O186" t="n">
         <v>0</v>
       </c>
@@ -28753,7 +29465,11 @@
         <v>0</v>
       </c>
       <c r="V186" t="inlineStr"/>
-      <c r="W186" t="inlineStr"/>
+      <c r="W186" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5325/649660/73c3cdd8-11a8-48ce-96d1-7968458a54f3.jpg</t>
+        </is>
+      </c>
       <c r="X186" t="n">
         <v>0</v>
       </c>
@@ -28881,7 +29597,11 @@
         <v>154374</v>
       </c>
       <c r="M187" t="inlineStr"/>
-      <c r="N187" t="inlineStr"/>
+      <c r="N187" t="inlineStr">
+        <is>
+          <t>1781976918568</t>
+        </is>
+      </c>
       <c r="O187" t="n">
         <v>0</v>
       </c>
@@ -28902,7 +29622,11 @@
         <v>0</v>
       </c>
       <c r="V187" t="inlineStr"/>
-      <c r="W187" t="inlineStr"/>
+      <c r="W187" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5325/649661/fa6d10c0-32ff-4d9f-8870-4f338cc3a080.jpg</t>
+        </is>
+      </c>
       <c r="X187" t="n">
         <v>0</v>
       </c>
@@ -29030,7 +29754,11 @@
         <v>154375</v>
       </c>
       <c r="M188" t="inlineStr"/>
-      <c r="N188" t="inlineStr"/>
+      <c r="N188" t="inlineStr">
+        <is>
+          <t>1781976789878</t>
+        </is>
+      </c>
       <c r="O188" t="n">
         <v>0</v>
       </c>
@@ -29051,7 +29779,11 @@
         <v>0</v>
       </c>
       <c r="V188" t="inlineStr"/>
-      <c r="W188" t="inlineStr"/>
+      <c r="W188" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5325/649662/5b3e686b-6cf4-4f2f-9bef-e2f19225fe00.jpg</t>
+        </is>
+      </c>
       <c r="X188" t="n">
         <v>0</v>
       </c>
@@ -29179,7 +29911,11 @@
         <v>154376</v>
       </c>
       <c r="M189" t="inlineStr"/>
-      <c r="N189" t="inlineStr"/>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>1781976797331</t>
+        </is>
+      </c>
       <c r="O189" t="n">
         <v>0</v>
       </c>
@@ -29200,7 +29936,11 @@
         <v>0</v>
       </c>
       <c r="V189" t="inlineStr"/>
-      <c r="W189" t="inlineStr"/>
+      <c r="W189" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5325/649663/8a743a8d-4bb6-4b52-9ee0-fb096d05a423.jpg</t>
+        </is>
+      </c>
       <c r="X189" t="n">
         <v>0</v>
       </c>
@@ -29328,7 +30068,11 @@
         <v>72830</v>
       </c>
       <c r="M190" t="inlineStr"/>
-      <c r="N190" t="inlineStr"/>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>1781976767139</t>
+        </is>
+      </c>
       <c r="O190" t="n">
         <v>0</v>
       </c>
@@ -29349,7 +30093,11 @@
         <v>0</v>
       </c>
       <c r="V190" t="inlineStr"/>
-      <c r="W190" t="inlineStr"/>
+      <c r="W190" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5326/72134/55cf203d-8a69-414e-b9f7-ee4a11783f74.jpg</t>
+        </is>
+      </c>
       <c r="X190" t="n">
         <v>0</v>
       </c>
@@ -29477,7 +30225,11 @@
         <v>72831</v>
       </c>
       <c r="M191" t="inlineStr"/>
-      <c r="N191" t="inlineStr"/>
+      <c r="N191" t="inlineStr">
+        <is>
+          <t>1781976758295</t>
+        </is>
+      </c>
       <c r="O191" t="n">
         <v>0</v>
       </c>
@@ -29498,7 +30250,11 @@
         <v>0</v>
       </c>
       <c r="V191" t="inlineStr"/>
-      <c r="W191" t="inlineStr"/>
+      <c r="W191" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5326/72135/3299ef7c-58ba-4205-af97-e137137941bd.jpg</t>
+        </is>
+      </c>
       <c r="X191" t="n">
         <v>0</v>
       </c>
@@ -29626,7 +30382,11 @@
         <v>72832</v>
       </c>
       <c r="M192" t="inlineStr"/>
-      <c r="N192" t="inlineStr"/>
+      <c r="N192" t="inlineStr">
+        <is>
+          <t>1781976979177</t>
+        </is>
+      </c>
       <c r="O192" t="n">
         <v>0</v>
       </c>
@@ -29647,7 +30407,11 @@
         <v>0</v>
       </c>
       <c r="V192" t="inlineStr"/>
-      <c r="W192" t="inlineStr"/>
+      <c r="W192" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5326/72136/10f48ffc-e0cf-456c-850e-deca15d1da85.jpg</t>
+        </is>
+      </c>
       <c r="X192" t="n">
         <v>0</v>
       </c>
@@ -29775,7 +30539,11 @@
         <v>72833</v>
       </c>
       <c r="M193" t="inlineStr"/>
-      <c r="N193" t="inlineStr"/>
+      <c r="N193" t="inlineStr">
+        <is>
+          <t>1781976824211</t>
+        </is>
+      </c>
       <c r="O193" t="n">
         <v>0</v>
       </c>
@@ -29796,7 +30564,11 @@
         <v>0</v>
       </c>
       <c r="V193" t="inlineStr"/>
-      <c r="W193" t="inlineStr"/>
+      <c r="W193" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5326/72137/5d545860-9405-4693-b8e3-56924e2893bc.jpg</t>
+        </is>
+      </c>
       <c r="X193" t="n">
         <v>0</v>
       </c>
@@ -29924,7 +30696,11 @@
         <v>72834</v>
       </c>
       <c r="M194" t="inlineStr"/>
-      <c r="N194" t="inlineStr"/>
+      <c r="N194" t="inlineStr">
+        <is>
+          <t>1781976933383</t>
+        </is>
+      </c>
       <c r="O194" t="n">
         <v>0</v>
       </c>
@@ -29945,7 +30721,11 @@
         <v>0</v>
       </c>
       <c r="V194" t="inlineStr"/>
-      <c r="W194" t="inlineStr"/>
+      <c r="W194" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5326/72138/a09214a6-8831-4033-9416-5be07b7eb1b8.jpg</t>
+        </is>
+      </c>
       <c r="X194" t="n">
         <v>0</v>
       </c>
@@ -30073,7 +30853,11 @@
         <v>72835</v>
       </c>
       <c r="M195" t="inlineStr"/>
-      <c r="N195" t="inlineStr"/>
+      <c r="N195" t="inlineStr">
+        <is>
+          <t>1781977057039</t>
+        </is>
+      </c>
       <c r="O195" t="n">
         <v>0</v>
       </c>
@@ -30094,7 +30878,11 @@
         <v>0</v>
       </c>
       <c r="V195" t="inlineStr"/>
-      <c r="W195" t="inlineStr"/>
+      <c r="W195" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5326/72139/c3b9796b-bcbc-4cdd-91b7-6f0738551d27.jpg</t>
+        </is>
+      </c>
       <c r="X195" t="n">
         <v>0</v>
       </c>
@@ -30222,7 +31010,11 @@
         <v>72836</v>
       </c>
       <c r="M196" t="inlineStr"/>
-      <c r="N196" t="inlineStr"/>
+      <c r="N196" t="inlineStr">
+        <is>
+          <t>1781976819622</t>
+        </is>
+      </c>
       <c r="O196" t="n">
         <v>0</v>
       </c>
@@ -30243,7 +31035,11 @@
         <v>0</v>
       </c>
       <c r="V196" t="inlineStr"/>
-      <c r="W196" t="inlineStr"/>
+      <c r="W196" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5326/72140/31a8e1ef-df90-4c0f-a81d-dffe6d5a2e49.jpg</t>
+        </is>
+      </c>
       <c r="X196" t="n">
         <v>0</v>
       </c>
@@ -30520,7 +31316,11 @@
         <v>72838</v>
       </c>
       <c r="M198" t="inlineStr"/>
-      <c r="N198" t="inlineStr"/>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>1781976808288</t>
+        </is>
+      </c>
       <c r="O198" t="n">
         <v>0</v>
       </c>
@@ -30541,7 +31341,11 @@
         <v>0</v>
       </c>
       <c r="V198" t="inlineStr"/>
-      <c r="W198" t="inlineStr"/>
+      <c r="W198" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5326/72142/70ca41c8-64d5-4fb6-8608-412d937ad039.jpg</t>
+        </is>
+      </c>
       <c r="X198" t="n">
         <v>0</v>
       </c>
@@ -30669,7 +31473,11 @@
         <v>72839</v>
       </c>
       <c r="M199" t="inlineStr"/>
-      <c r="N199" t="inlineStr"/>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>1781976930445</t>
+        </is>
+      </c>
       <c r="O199" t="n">
         <v>0</v>
       </c>
@@ -30690,7 +31498,11 @@
         <v>0</v>
       </c>
       <c r="V199" t="inlineStr"/>
-      <c r="W199" t="inlineStr"/>
+      <c r="W199" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5326/72143/ab1c0ba3-2ebe-4cdf-a507-6e8a170edbf1.jpg</t>
+        </is>
+      </c>
       <c r="X199" t="n">
         <v>0</v>
       </c>
@@ -30818,7 +31630,11 @@
         <v>72840</v>
       </c>
       <c r="M200" t="inlineStr"/>
-      <c r="N200" t="inlineStr"/>
+      <c r="N200" t="inlineStr">
+        <is>
+          <t>1781976985755</t>
+        </is>
+      </c>
       <c r="O200" t="n">
         <v>0</v>
       </c>
@@ -30839,7 +31655,11 @@
         <v>0</v>
       </c>
       <c r="V200" t="inlineStr"/>
-      <c r="W200" t="inlineStr"/>
+      <c r="W200" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5326/72144/5673191c-53f4-4aec-876f-1c7b818a3c79.jpg</t>
+        </is>
+      </c>
       <c r="X200" t="n">
         <v>0</v>
       </c>
@@ -30967,7 +31787,11 @@
         <v>154377</v>
       </c>
       <c r="M201" t="inlineStr"/>
-      <c r="N201" t="inlineStr"/>
+      <c r="N201" t="inlineStr">
+        <is>
+          <t>1781976752810</t>
+        </is>
+      </c>
       <c r="O201" t="n">
         <v>0</v>
       </c>
@@ -30988,7 +31812,11 @@
         <v>0</v>
       </c>
       <c r="V201" t="inlineStr"/>
-      <c r="W201" t="inlineStr"/>
+      <c r="W201" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2990/22/468/5326/649664/f5638765-6302-4db2-a636-44fe420183eb.jpg</t>
+        </is>
+      </c>
       <c r="X201" t="n">
         <v>0</v>
       </c>
@@ -31457,22 +32285,22 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -31490,7 +32318,7 @@
         <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="P4" t="n">
         <v>0</v>
@@ -31665,22 +32493,22 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1500</v>
+        <v>2250</v>
       </c>
       <c r="E6" t="n">
-        <v>72</v>
+        <v>126</v>
       </c>
       <c r="F6" t="n">
         <v>4</v>
       </c>
       <c r="G6" t="n">
-        <v>72</v>
+        <v>126</v>
       </c>
       <c r="H6" t="n">
-        <v>1500</v>
+        <v>2250</v>
       </c>
       <c r="I6" t="n">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="J6" t="n">
         <v>0</v>
@@ -31698,7 +32526,7 @@
         <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>64</v>
+        <v>116</v>
       </c>
       <c r="P6" t="n">
         <v>0</v>
@@ -31716,7 +32544,7 @@
         <v>0</v>
       </c>
       <c r="U6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="V6" t="n">
         <v>0</v>
@@ -32455,22 +33283,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3083</v>
+        <v>4583</v>
       </c>
       <c r="D2" t="n">
-        <v>184</v>
+        <v>273</v>
       </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F2" t="n">
-        <v>182</v>
+        <v>271</v>
       </c>
       <c r="G2" t="n">
-        <v>2709</v>
+        <v>4209</v>
       </c>
       <c r="H2" t="n">
-        <v>178</v>
+        <v>266</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -32488,7 +33316,7 @@
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>169</v>
+        <v>255</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -32506,7 +33334,7 @@
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
@@ -32715,22 +33543,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3083</v>
+        <v>4583</v>
       </c>
       <c r="C2" t="n">
-        <v>184</v>
+        <v>273</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>182</v>
+        <v>271</v>
       </c>
       <c r="F2" t="n">
-        <v>2709</v>
+        <v>4209</v>
       </c>
       <c r="G2" t="n">
-        <v>178</v>
+        <v>266</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -32748,7 +33576,7 @@
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>169</v>
+        <v>255</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
@@ -32766,7 +33594,7 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="T2" t="n">
         <v>0</v>

</xml_diff>